<commit_message>
update files w/ SYVBT values BAADTbVT, TTS, SYVBT
</commit_message>
<xml_diff>
--- a/InputData/trans/TTS/Transportation Technology Shareweights.xlsx
+++ b/InputData/trans/TTS/Transportation Technology Shareweights.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\trans\TTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872A5FAF-3508-41B4-9C6A-91448C22D520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63F1C5A-A64A-4FB6-A25E-9AF5B9620F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="360" windowWidth="17490" windowHeight="9240" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -10803,115 +10803,115 @@
       </c>
       <c r="B3">
         <f>Data!I25</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="C3">
         <f>Data!J25</f>
-        <v>0.30697688955366859</v>
+        <v>0.30697688951733509</v>
       </c>
       <c r="D3">
         <f>Data!K25</f>
-        <v>0.30769353631198043</v>
+        <v>0.30769353627583379</v>
       </c>
       <c r="E3">
         <f>Data!L25</f>
-        <v>0.30864929954161624</v>
+        <v>0.30864929950571873</v>
       </c>
       <c r="F3">
         <f>Data!M25</f>
-        <v>0.30991873901568157</v>
+        <v>0.30991873898011502</v>
       </c>
       <c r="G3">
         <f>Data!N25</f>
-        <v>0.31159563622314707</v>
+        <v>0.31159563618801772</v>
       </c>
       <c r="H3">
         <f>Data!O25</f>
-        <v>0.31379489609651995</v>
+        <v>0.31379489606196392</v>
       </c>
       <c r="I3">
         <f>Data!P25</f>
-        <v>0.31665218169291087</v>
+        <v>0.31665218165909981</v>
       </c>
       <c r="J3">
         <f>Data!Q25</f>
-        <v>0.32031926321671017</v>
+        <v>0.32031926318385517</v>
       </c>
       <c r="K3">
         <f>Data!R25</f>
-        <v>0.32495249513093305</v>
+        <v>0.32495249509928592</v>
       </c>
       <c r="L3">
         <f>Data!S25</f>
-        <v>0.33069193089989313</v>
+        <v>0.33069193086974236</v>
       </c>
       <c r="M3">
         <f>Data!T25</f>
-        <v>0.33763022578538127</v>
+        <v>0.33763022575703938</v>
       </c>
       <c r="N3">
         <f>Data!U25</f>
-        <v>0.34577450263754761</v>
+        <v>0.34577450261132897</v>
       </c>
       <c r="O3">
         <f>Data!V25</f>
-        <v>0.3550105126051174</v>
+        <v>0.35501051258130667</v>
       </c>
       <c r="P3">
         <f>Data!W25</f>
-        <v>0.36508401650950512</v>
+        <v>0.36508401648832067</v>
       </c>
       <c r="Q3">
         <f>Data!X25</f>
-        <v>0.37561423811298911</v>
+        <v>0.37561423809454991</v>
       </c>
       <c r="R3">
         <f>Data!Y25</f>
-        <v>0.38614445971647304</v>
+        <v>0.38614445970077915</v>
       </c>
       <c r="S3">
         <f>Data!Z25</f>
-        <v>0.39621796362086076</v>
+        <v>0.39621796360779316</v>
       </c>
       <c r="T3">
         <f>Data!AA25</f>
-        <v>0.40545397358843055</v>
+        <v>0.40545397357777085</v>
       </c>
       <c r="U3">
         <f>Data!AB25</f>
-        <v>0.41359825044059684</v>
+        <v>0.41359825043206044</v>
       </c>
       <c r="V3">
         <f>Data!AC25</f>
-        <v>0.42053654532608503</v>
+        <v>0.42053654531935747</v>
       </c>
       <c r="W3">
         <f>Data!AD25</f>
-        <v>0.42627598109504511</v>
+        <v>0.4262759810898139</v>
       </c>
       <c r="X3">
         <f>Data!AE25</f>
-        <v>0.43090921300926799</v>
+        <v>0.43090921300524465</v>
       </c>
       <c r="Y3">
         <f>Data!AF25</f>
-        <v>0.43457629453306729</v>
+        <v>0.43457629453000002</v>
       </c>
       <c r="Z3">
         <f>Data!AG25</f>
-        <v>0.43743358012945821</v>
+        <v>0.43743358012713585</v>
       </c>
       <c r="AA3">
         <f>Data!AH25</f>
-        <v>0.43963284000283109</v>
+        <v>0.43963284000108216</v>
       </c>
       <c r="AB3">
         <f>Data!AI25</f>
-        <v>0.44130973721029659</v>
+        <v>0.44130973720898481</v>
       </c>
       <c r="AC3">
         <f>Data!AJ25</f>
-        <v>0.44257917668436197</v>
+        <v>0.44257917668338109</v>
       </c>
       <c r="AD3">
         <f>Data!AK25</f>
@@ -10928,115 +10928,115 @@
       </c>
       <c r="B4">
         <f>Data!I26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="C4">
         <f>Data!J26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="D4">
         <f>Data!K26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="E4">
         <f>Data!L26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="F4">
         <f>Data!M26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="G4">
         <f>Data!N26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="H4">
         <f>Data!O26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="I4">
         <f>Data!P26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="J4">
         <f>Data!Q26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="K4">
         <f>Data!R26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="L4">
         <f>Data!S26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="M4">
         <f>Data!T26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="N4">
         <f>Data!U26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="O4">
         <f>Data!V26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="P4">
         <f>Data!W26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="Q4">
         <f>Data!X26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="R4">
         <f>Data!Y26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="S4">
         <f>Data!Z26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="T4">
         <f>Data!AA26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="U4">
         <f>Data!AB26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="V4">
         <f>Data!AC26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="W4">
         <f>Data!AD26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="X4">
         <f>Data!AE26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="Y4">
         <f>Data!AF26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="Z4">
         <f>Data!AG26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AA4">
         <f>Data!AH26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AB4">
         <f>Data!AI26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AC4">
         <f>Data!AJ26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AD4">
         <f>Data!AK26</f>
@@ -11303,115 +11303,115 @@
       </c>
       <c r="B7">
         <f>Data!I29</f>
-        <v>0.12967078621379674</v>
+        <v>0.12967078621466466</v>
       </c>
       <c r="C7">
         <f>Data!J29</f>
-        <v>0.12967078621379358</v>
+        <v>0.12967078621466044</v>
       </c>
       <c r="D7">
         <f>Data!K29</f>
-        <v>0.14540917710224477</v>
+        <v>0.14540917710321821</v>
       </c>
       <c r="E7">
         <f>Data!L29</f>
-        <v>0.16114756799069241</v>
+        <v>0.16114756799177243</v>
       </c>
       <c r="F7">
         <f>Data!M29</f>
-        <v>0.1768859588791436</v>
+        <v>0.17688595888033021</v>
       </c>
       <c r="G7">
         <f>Data!N29</f>
-        <v>0.19262434976759479</v>
+        <v>0.19262434976888443</v>
       </c>
       <c r="H7">
         <f>Data!O29</f>
-        <v>0.20836274065604599</v>
+        <v>0.2083627406574422</v>
       </c>
       <c r="I7">
         <f>Data!P29</f>
-        <v>0.22410113154449718</v>
+        <v>0.22410113154599642</v>
       </c>
       <c r="J7">
         <f>Data!Q29</f>
-        <v>0.23983952243294837</v>
+        <v>0.2398395224345542</v>
       </c>
       <c r="K7">
         <f>Data!R29</f>
-        <v>0.25557791332139956</v>
+        <v>0.25557791332310842</v>
       </c>
       <c r="L7">
         <f>Data!S29</f>
-        <v>0.27131630420985076</v>
+        <v>0.27131630421166619</v>
       </c>
       <c r="M7">
         <f>Data!T29</f>
-        <v>0.28705469509830195</v>
+        <v>0.28705469510022041</v>
       </c>
       <c r="N7">
         <f>Data!U29</f>
-        <v>0.30279308598675314</v>
+        <v>0.30279308598877819</v>
       </c>
       <c r="O7">
         <f>Data!V29</f>
-        <v>0.31853147687520433</v>
+        <v>0.31853147687733596</v>
       </c>
       <c r="P7">
         <f>Data!W29</f>
-        <v>0.33426986776365553</v>
+        <v>0.33426986776589374</v>
       </c>
       <c r="Q7">
         <f>Data!X29</f>
-        <v>0.35000825865210672</v>
+        <v>0.3500082586544444</v>
       </c>
       <c r="R7">
         <f>Data!Y29</f>
-        <v>0.36574664954055791</v>
+        <v>0.36574664954300218</v>
       </c>
       <c r="S7">
         <f>Data!Z29</f>
-        <v>0.381485040429002</v>
+        <v>0.38148504043155995</v>
       </c>
       <c r="T7">
         <f>Data!AA29</f>
-        <v>0.39722343131745319</v>
+        <v>0.39722343132011773</v>
       </c>
       <c r="U7">
         <f>Data!AB29</f>
-        <v>0.41296182220590438</v>
+        <v>0.41296182220866839</v>
       </c>
       <c r="V7">
         <f>Data!AC29</f>
-        <v>0.42870021309435558</v>
+        <v>0.42870021309722617</v>
       </c>
       <c r="W7">
         <f>Data!AD29</f>
-        <v>0.44443860398280677</v>
+        <v>0.44443860398578394</v>
       </c>
       <c r="X7">
         <f>Data!AE29</f>
-        <v>0.46017699487125796</v>
+        <v>0.46017699487434172</v>
       </c>
       <c r="Y7">
         <f>Data!AF29</f>
-        <v>0.47591538575970915</v>
+        <v>0.47591538576289238</v>
       </c>
       <c r="Z7">
         <f>Data!AG29</f>
-        <v>0.49165377664816035</v>
+        <v>0.49165377665145016</v>
       </c>
       <c r="AA7">
         <f>Data!AH29</f>
-        <v>0.50739216753661154</v>
+        <v>0.50739216754000793</v>
       </c>
       <c r="AB7">
         <f>Data!AI29</f>
-        <v>0.52313055842506273</v>
+        <v>0.52313055842856571</v>
       </c>
       <c r="AC7">
         <f>Data!AJ29</f>
-        <v>0.53886894931351392</v>
+        <v>0.53886894931712348</v>
       </c>
       <c r="AD7">
         <f>Data!AK29</f>
@@ -11428,115 +11428,115 @@
       </c>
       <c r="B8">
         <f>Data!I30</f>
-        <v>1.0880490304811035E-4</v>
+        <v>1.088049030359405E-4</v>
       </c>
       <c r="C8">
         <f>Data!J30</f>
-        <v>8.4589900062574685E-4</v>
+        <v>8.4589900061375677E-4</v>
       </c>
       <c r="D8">
         <f>Data!K30</f>
-        <v>1.0986614672101446E-3</v>
+        <v>1.0986614671982162E-3</v>
       </c>
       <c r="E8">
         <f>Data!L30</f>
-        <v>1.4357606985839016E-3</v>
+        <v>1.4357606985720554E-3</v>
       </c>
       <c r="F8">
         <f>Data!M30</f>
-        <v>1.8834940468798042E-3</v>
+        <v>1.883494046868067E-3</v>
       </c>
       <c r="G8">
         <f>Data!N30</f>
-        <v>2.4749383943933924E-3</v>
+        <v>2.4749383943817997E-3</v>
       </c>
       <c r="H8">
         <f>Data!O30</f>
-        <v>3.2506208959975401E-3</v>
+        <v>3.2506208959861365E-3</v>
       </c>
       <c r="I8">
         <f>Data!P30</f>
-        <v>4.2583901305659581E-3</v>
+        <v>4.2583901305548004E-3</v>
       </c>
       <c r="J8">
         <f>Data!Q30</f>
-        <v>5.5517756937757106E-3</v>
+        <v>5.5517756937648686E-3</v>
       </c>
       <c r="K8">
         <f>Data!R30</f>
-        <v>7.185924056708733E-3</v>
+        <v>7.1859240566982891E-3</v>
       </c>
       <c r="L8">
         <f>Data!S30</f>
-        <v>9.2102323019346774E-3</v>
+        <v>9.210232301924727E-3</v>
       </c>
       <c r="M8">
         <f>Data!T30</f>
-        <v>1.1657380089607801E-2</v>
+        <v>1.1657380089598447E-2</v>
       </c>
       <c r="N8">
         <f>Data!U30</f>
-        <v>1.452987966045502E-2</v>
+        <v>1.4529879660446367E-2</v>
       </c>
       <c r="O8">
         <f>Data!V30</f>
-        <v>1.7787435260511523E-2</v>
+        <v>1.7787435260503668E-2</v>
       </c>
       <c r="P8">
         <f>Data!W30</f>
-        <v>2.1340376321765452E-2</v>
+        <v>2.1340376321758465E-2</v>
       </c>
       <c r="Q8">
         <f>Data!X30</f>
-        <v>2.5054402451524054E-2</v>
+        <v>2.5054402451517972E-2</v>
       </c>
       <c r="R8">
         <f>Data!Y30</f>
-        <v>2.8768428581282656E-2</v>
+        <v>2.876842858127748E-2</v>
       </c>
       <c r="S8">
         <f>Data!Z30</f>
-        <v>3.2321369642536582E-2</v>
+        <v>3.2321369642532273E-2</v>
       </c>
       <c r="T8">
         <f>Data!AA30</f>
-        <v>3.5578925242593096E-2</v>
+        <v>3.5578925242589578E-2</v>
       </c>
       <c r="U8">
         <f>Data!AB30</f>
-        <v>3.8451424813440313E-2</v>
+        <v>3.8451424813437496E-2</v>
       </c>
       <c r="V8">
         <f>Data!AC30</f>
-        <v>4.0898572601113438E-2</v>
+        <v>4.0898572601111217E-2</v>
       </c>
       <c r="W8">
         <f>Data!AD30</f>
-        <v>4.2922880846339384E-2</v>
+        <v>4.2922880846337656E-2</v>
       </c>
       <c r="X8">
         <f>Data!AE30</f>
-        <v>4.4557029209272403E-2</v>
+        <v>4.4557029209271078E-2</v>
       </c>
       <c r="Y8">
         <f>Data!AF30</f>
-        <v>4.5850414772482161E-2</v>
+        <v>4.5850414772481148E-2</v>
       </c>
       <c r="Z8">
         <f>Data!AG30</f>
-        <v>4.6858184007050573E-2</v>
+        <v>4.6858184007049809E-2</v>
       </c>
       <c r="AA8">
         <f>Data!AH30</f>
-        <v>4.7633866508654726E-2</v>
+        <v>4.763386650865415E-2</v>
       </c>
       <c r="AB8">
         <f>Data!AI30</f>
-        <v>4.822531085616831E-2</v>
+        <v>4.822531085616788E-2</v>
       </c>
       <c r="AC8">
         <f>Data!AJ30</f>
-        <v>4.8673044204464208E-2</v>
+        <v>4.8673044204463882E-2</v>
       </c>
       <c r="AD8">
         <f>Data!AK30</f>
@@ -14742,115 +14742,115 @@
       </c>
       <c r="B2">
         <f>Data!I52</f>
-        <v>0.93664816809218165</v>
+        <v>0.93664816810144857</v>
       </c>
       <c r="C2">
         <f>Data!J52</f>
-        <v>0.93758413006461472</v>
+        <v>0.93758413007374464</v>
       </c>
       <c r="D2">
         <f>Data!K52</f>
-        <v>0.93790508780604664</v>
+        <v>0.93790508781512971</v>
       </c>
       <c r="E2">
         <f>Data!L52</f>
-        <v>0.93833313635851656</v>
+        <v>0.93833313636753701</v>
       </c>
       <c r="F2">
         <f>Data!M52</f>
-        <v>0.93890166809574294</v>
+        <v>0.93890166810468023</v>
       </c>
       <c r="G2">
         <f>Data!N52</f>
-        <v>0.93965268403780833</v>
+        <v>0.93965268404663582</v>
       </c>
       <c r="H2">
         <f>Data!O52</f>
-        <v>0.94063764555977569</v>
+        <v>0.94063764556845908</v>
       </c>
       <c r="I2">
         <f>Data!P52</f>
-        <v>0.94191731077978458</v>
+        <v>0.94191731078828078</v>
       </c>
       <c r="J2">
         <f>Data!Q52</f>
-        <v>0.94355965157024346</v>
+        <v>0.94355965157849941</v>
       </c>
       <c r="K2">
         <f>Data!R52</f>
-        <v>0.94563469291170243</v>
+        <v>0.94563469291965474</v>
       </c>
       <c r="L2">
         <f>Data!S52</f>
-        <v>0.94820515921205761</v>
+        <v>0.94820515921963411</v>
       </c>
       <c r="M2">
         <f>Data!T52</f>
-        <v>0.95131254709877777</v>
+        <v>0.95131254710589963</v>
       </c>
       <c r="N2">
         <f>Data!U52</f>
-        <v>0.95496004661475364</v>
+        <v>0.95496004662134204</v>
       </c>
       <c r="O2">
         <f>Data!V52</f>
-        <v>0.95909649021776056</v>
+        <v>0.95909649022374377</v>
       </c>
       <c r="P2">
         <f>Data!W52</f>
-        <v>0.96360801423424369</v>
+        <v>0.96360801423956699</v>
       </c>
       <c r="Q2">
         <f>Data!X52</f>
-        <v>0.96832408404609083</v>
+        <v>0.96832408405072434</v>
       </c>
       <c r="R2">
         <f>Data!Y52</f>
-        <v>0.97304015385793796</v>
+        <v>0.97304015386188158</v>
       </c>
       <c r="S2">
         <f>Data!Z52</f>
-        <v>0.9775516778744211</v>
+        <v>0.97755167787770481</v>
       </c>
       <c r="T2">
         <f>Data!AA52</f>
-        <v>0.98168812147742801</v>
+        <v>0.98168812148010653</v>
       </c>
       <c r="U2">
         <f>Data!AB52</f>
-        <v>0.98533562099340388</v>
+        <v>0.98533562099554894</v>
       </c>
       <c r="V2">
         <f>Data!AC52</f>
-        <v>0.98844300888012404</v>
+        <v>0.98844300888181458</v>
       </c>
       <c r="W2">
         <f>Data!AD52</f>
-        <v>0.99101347518047922</v>
+        <v>0.99101347518179383</v>
       </c>
       <c r="X2">
         <f>Data!AE52</f>
-        <v>0.99308851652193819</v>
+        <v>0.99308851652294916</v>
       </c>
       <c r="Y2">
         <f>Data!AF52</f>
-        <v>0.99473085731239708</v>
+        <v>0.99473085731316779</v>
       </c>
       <c r="Z2">
         <f>Data!AG52</f>
-        <v>0.99601052253240596</v>
+        <v>0.9960105225329895</v>
       </c>
       <c r="AA2">
         <f>Data!AH52</f>
-        <v>0.99699548405437333</v>
+        <v>0.99699548405481275</v>
       </c>
       <c r="AB2">
         <f>Data!AI52</f>
-        <v>0.99774649999643872</v>
+        <v>0.99774649999676845</v>
       </c>
       <c r="AC2">
         <f>Data!AJ52</f>
-        <v>0.99831503173366509</v>
+        <v>0.99831503173391156</v>
       </c>
       <c r="AD2">
         <f>Data!AK52</f>
@@ -15117,111 +15117,111 @@
       </c>
       <c r="B5">
         <f>Data!I55</f>
-        <v>6.3351831907818346E-2</v>
+        <v>6.3351831898551425E-2</v>
       </c>
       <c r="C5">
         <f>Data!J55</f>
-        <v>6.3351831907809242E-2</v>
+        <v>6.3351831898543765E-2</v>
       </c>
       <c r="D5">
         <f>Data!K55</f>
-        <v>9.9376761449818218E-2</v>
+        <v>9.9376761440908012E-2</v>
       </c>
       <c r="E5">
         <f>Data!L55</f>
-        <v>0.13540169099182719</v>
+        <v>0.13540169098327226</v>
       </c>
       <c r="F5">
         <f>Data!M55</f>
-        <v>0.17142662053383617</v>
+        <v>0.17142662052563651</v>
       </c>
       <c r="G5">
         <f>Data!N55</f>
-        <v>0.20745155007584515</v>
+        <v>0.20745155006800076</v>
       </c>
       <c r="H5">
         <f>Data!O55</f>
-        <v>0.24347647961785412</v>
+        <v>0.243476479610365</v>
       </c>
       <c r="I5">
         <f>Data!P55</f>
-        <v>0.2795014091598631</v>
+        <v>0.27950140915272925</v>
       </c>
       <c r="J5">
         <f>Data!Q55</f>
-        <v>0.31552633870185787</v>
+        <v>0.3155263386950935</v>
       </c>
       <c r="K5">
         <f>Data!R55</f>
-        <v>0.35155126824386684</v>
+        <v>0.35155126823745775</v>
       </c>
       <c r="L5">
         <f>Data!S55</f>
-        <v>0.38757619778587582</v>
+        <v>0.387576197779822</v>
       </c>
       <c r="M5">
         <f>Data!T55</f>
-        <v>0.4236011273278848</v>
+        <v>0.42360112732218624</v>
       </c>
       <c r="N5">
         <f>Data!U55</f>
-        <v>0.45962605686989377</v>
+        <v>0.45962605686455049</v>
       </c>
       <c r="O5">
         <f>Data!V55</f>
-        <v>0.49565098641190275</v>
+        <v>0.49565098640691474</v>
       </c>
       <c r="P5">
         <f>Data!W55</f>
-        <v>0.53167591595391173</v>
+        <v>0.53167591594927899</v>
       </c>
       <c r="Q5">
         <f>Data!X55</f>
-        <v>0.56770084549590649</v>
+        <v>0.56770084549164324</v>
       </c>
       <c r="R5">
         <f>Data!Y55</f>
-        <v>0.60372577503791547</v>
+        <v>0.60372577503400748</v>
       </c>
       <c r="S5">
         <f>Data!Z55</f>
-        <v>0.63975070457992445</v>
+        <v>0.63975070457635752</v>
       </c>
       <c r="T5">
         <f>Data!AA55</f>
-        <v>0.67577563412193342</v>
+        <v>0.67577563411872177</v>
       </c>
       <c r="U5">
         <f>Data!AB55</f>
-        <v>0.7118005636639424</v>
+        <v>0.71180056366108602</v>
       </c>
       <c r="V5">
         <f>Data!AC55</f>
-        <v>0.74782549320595137</v>
+        <v>0.74782549320345026</v>
       </c>
       <c r="W5">
         <f>Data!AD55</f>
-        <v>0.78385042274796035</v>
+        <v>0.78385042274581451</v>
       </c>
       <c r="X5">
         <f>Data!AE55</f>
-        <v>0.81987535228995512</v>
+        <v>0.81987535228817876</v>
       </c>
       <c r="Y5">
         <f>Data!AF55</f>
-        <v>0.85590028183196409</v>
+        <v>0.85590028183054301</v>
       </c>
       <c r="Z5">
         <f>Data!AG55</f>
-        <v>0.89192521137397307</v>
+        <v>0.89192521137290726</v>
       </c>
       <c r="AA5">
         <f>Data!AH55</f>
-        <v>0.92795014091598205</v>
+        <v>0.9279501409152715</v>
       </c>
       <c r="AB5">
         <f>Data!AI55</f>
-        <v>0.96397507045799102</v>
+        <v>0.96397507045763575</v>
       </c>
       <c r="AC5">
         <f>Data!AJ55</f>
@@ -52302,188 +52302,188 @@
     <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" t="s">
         <v>111</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2">
         <v>2799214</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2">
         <v>16648</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2">
         <v>256819978</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2">
         <v>1348635</v>
       </c>
-      <c r="F2" s="5">
-        <v>1130472.0000000002</v>
-      </c>
-      <c r="G2" s="5">
+      <c r="F2">
+        <v>1130472</v>
+      </c>
+      <c r="G2">
         <v>16384</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2">
         <v>15809</v>
       </c>
       <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3">
         <v>300</v>
       </c>
-      <c r="C3" s="5">
-        <v>123405.86316307285</v>
-      </c>
-      <c r="D3" s="5">
-        <v>98369.804893824577</v>
-      </c>
-      <c r="E3" s="5">
-        <v>703911.92875736777</v>
-      </c>
-      <c r="F3" s="5">
-        <v>0</v>
-      </c>
-      <c r="G3" s="5">
-        <v>41837.429476286045</v>
-      </c>
-      <c r="H3" s="5">
-        <v>105.31556700313551</v>
+      <c r="C3">
+        <v>123405.86320000001</v>
+      </c>
+      <c r="D3">
+        <v>98369.804889999999</v>
+      </c>
+      <c r="E3">
+        <v>703911.92879999999</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>41837.429479999999</v>
+      </c>
+      <c r="H3">
+        <v>105.315567</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="24"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="5">
-        <v>0</v>
-      </c>
-      <c r="C4" s="5">
-        <v>0</v>
-      </c>
-      <c r="D4" s="5">
-        <v>0</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>0</v>
-      </c>
-      <c r="G4" s="5">
-        <v>0</v>
-      </c>
-      <c r="H4" s="5">
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
-        <v>2563.6060360683009</v>
-      </c>
-      <c r="C5" s="5">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5">
-        <v>173.39396393169866</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="5">
+      <c r="B5">
+        <v>2563.6060360000001</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>173.39396389999999</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="5">
-        <v>0</v>
-      </c>
-      <c r="C6" s="5">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5">
-        <v>10231405.018379824</v>
-      </c>
-      <c r="E6" s="5">
-        <v>2473594.5350763109</v>
-      </c>
-      <c r="F6" s="5">
-        <v>0</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0</v>
-      </c>
-      <c r="H6" s="5">
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>10231405.02</v>
+      </c>
+      <c r="E6">
+        <v>2473594.5350000001</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="5">
-        <v>0</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5">
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
         <v>9516910</v>
       </c>
-      <c r="E7" s="5">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5">
-        <v>0</v>
-      </c>
-      <c r="H7" s="5">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>0</v>
       </c>
     </row>
@@ -62085,7 +62085,7 @@
       </c>
       <c r="E25" s="22">
         <f>'SYVbT-passenger'!D3/SUM('SYVbT-passenger'!3:3)*3</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="F25" s="22">
         <f>F32*3</f>
@@ -62097,115 +62097,115 @@
       </c>
       <c r="I25" s="22">
         <f t="shared" si="1"/>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="J25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,J$9))</f>
-        <v>0.30697688955366859</v>
+        <v>0.30697688951733509</v>
       </c>
       <c r="K25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,K$9))</f>
-        <v>0.30769353631198043</v>
+        <v>0.30769353627583379</v>
       </c>
       <c r="L25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,L$9))</f>
-        <v>0.30864929954161624</v>
+        <v>0.30864929950571873</v>
       </c>
       <c r="M25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,M$9))</f>
-        <v>0.30991873901568157</v>
+        <v>0.30991873898011502</v>
       </c>
       <c r="N25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,N$9))</f>
-        <v>0.31159563622314707</v>
+        <v>0.31159563618801772</v>
       </c>
       <c r="O25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,O$9))</f>
-        <v>0.31379489609651995</v>
+        <v>0.31379489606196392</v>
       </c>
       <c r="P25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,P$9))</f>
-        <v>0.31665218169291087</v>
+        <v>0.31665218165909981</v>
       </c>
       <c r="Q25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,Q$9))</f>
-        <v>0.32031926321671017</v>
+        <v>0.32031926318385517</v>
       </c>
       <c r="R25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,R$9))</f>
-        <v>0.32495249513093305</v>
+        <v>0.32495249509928592</v>
       </c>
       <c r="S25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,S$9))</f>
-        <v>0.33069193089989313</v>
+        <v>0.33069193086974236</v>
       </c>
       <c r="T25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,T$9))</f>
-        <v>0.33763022578538127</v>
+        <v>0.33763022575703938</v>
       </c>
       <c r="U25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,U$9))</f>
-        <v>0.34577450263754761</v>
+        <v>0.34577450261132897</v>
       </c>
       <c r="V25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,V$9))</f>
-        <v>0.3550105126051174</v>
+        <v>0.35501051258130667</v>
       </c>
       <c r="W25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,W$9))</f>
-        <v>0.36508401650950512</v>
+        <v>0.36508401648832067</v>
       </c>
       <c r="X25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,X$9))</f>
-        <v>0.37561423811298911</v>
+        <v>0.37561423809454991</v>
       </c>
       <c r="Y25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,Y$9))</f>
-        <v>0.38614445971647304</v>
+        <v>0.38614445970077915</v>
       </c>
       <c r="Z25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,Z$9))</f>
-        <v>0.39621796362086076</v>
+        <v>0.39621796360779316</v>
       </c>
       <c r="AA25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AA$9))</f>
-        <v>0.40545397358843055</v>
+        <v>0.40545397357777085</v>
       </c>
       <c r="AB25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AB$9))</f>
-        <v>0.41359825044059684</v>
+        <v>0.41359825043206044</v>
       </c>
       <c r="AC25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AC$9))</f>
-        <v>0.42053654532608503</v>
+        <v>0.42053654531935747</v>
       </c>
       <c r="AD25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AD$9))</f>
-        <v>0.42627598109504511</v>
+        <v>0.4262759810898139</v>
       </c>
       <c r="AE25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AE$9))</f>
-        <v>0.43090921300926799</v>
+        <v>0.43090921300524465</v>
       </c>
       <c r="AF25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AF$9))</f>
-        <v>0.43457629453306729</v>
+        <v>0.43457629453000002</v>
       </c>
       <c r="AG25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AG$9))</f>
-        <v>0.43743358012945821</v>
+        <v>0.43743358012713585</v>
       </c>
       <c r="AH25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AH$9))</f>
-        <v>0.43963284000283109</v>
+        <v>0.43963284000108216</v>
       </c>
       <c r="AI25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AI$9))</f>
-        <v>0.44130973721029659</v>
+        <v>0.44130973720898481</v>
       </c>
       <c r="AJ25">
         <f>IF($G25="s-curve",$E25+($F25-$E25)*$I$2/(1+EXP($I$3*(COUNT($I$9:AJ$9)+$I$4))),TREND($E25:$F25,$E$9:$F$9,AJ$9))</f>
-        <v>0.44257917668436197</v>
+        <v>0.44257917668338109</v>
       </c>
     </row>
     <row r="26" spans="1:36" x14ac:dyDescent="0.25">
@@ -62214,11 +62214,11 @@
       </c>
       <c r="E26" s="22">
         <f>'SYVbT-passenger'!D3/SUM('SYVbT-passenger'!3:3)*3</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="F26" s="22">
         <f>E26</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="G26" s="7" t="str">
         <f>IF(E26=F26,"n/a",IF(OR(C26="battery electric vehicle",C26="natural gas vehicle",C26="plugin hybrid vehicle"),"s-curve","linear"))</f>
@@ -62226,115 +62226,115 @@
       </c>
       <c r="I26" s="22">
         <f t="shared" si="1"/>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="J26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,J$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="K26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,K$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="L26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,L$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="M26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,M$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="N26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,N$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="O26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,O$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="P26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,P$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="Q26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,Q$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="R26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,R$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="S26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,S$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="T26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,T$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="U26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,U$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="V26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,V$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="W26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,W$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="X26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,X$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="Y26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,Y$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="Z26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,Z$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AA26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AA$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AB26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AB$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AC26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AC$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AD26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AD$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AE26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AE$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AF26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AF$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AG26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AG$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AH26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AH$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AI26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AI$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
       <c r="AJ26">
         <f>IF($G26="s-curve",$E26+($F26-$E26)*$I$2/(1+EXP($I$3*(COUNT($I$9:AJ$9)+$I$4))),TREND($E26:$F26,$E$9:$F$9,AJ$9))</f>
-        <v>0.30488703775431764</v>
+        <v>0.3048870377174393</v>
       </c>
     </row>
     <row r="27" spans="1:36" x14ac:dyDescent="0.25">
@@ -62599,11 +62599,11 @@
       </c>
       <c r="E29" s="22">
         <f>'SYVbT-passenger'!G3/SUM('SYVbT-passenger'!3:3)*3</f>
-        <v>0.12967078621379674</v>
+        <v>0.12967078621466466</v>
       </c>
       <c r="F29" s="22">
         <f>F36*($E$29/$E$36)*3</f>
-        <v>0.53886894931351725</v>
+        <v>0.53886894931712415</v>
       </c>
       <c r="G29" s="7" t="str">
         <f>IF(E29=F29,"n/a",IF(OR(C29="battery electric vehicle",C29="natural gas vehicle",C29="plugin hybrid vehicle",C29="hydrogen vehicle"),"s-curve","linear"))</f>
@@ -62611,115 +62611,115 @@
       </c>
       <c r="I29" s="22">
         <f t="shared" si="1"/>
-        <v>0.12967078621379674</v>
+        <v>0.12967078621466466</v>
       </c>
       <c r="J29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,J$9))</f>
-        <v>0.12967078621379358</v>
+        <v>0.12967078621466044</v>
       </c>
       <c r="K29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,K$9))</f>
-        <v>0.14540917710224477</v>
+        <v>0.14540917710321821</v>
       </c>
       <c r="L29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,L$9))</f>
-        <v>0.16114756799069241</v>
+        <v>0.16114756799177243</v>
       </c>
       <c r="M29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,M$9))</f>
-        <v>0.1768859588791436</v>
+        <v>0.17688595888033021</v>
       </c>
       <c r="N29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,N$9))</f>
-        <v>0.19262434976759479</v>
+        <v>0.19262434976888443</v>
       </c>
       <c r="O29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,O$9))</f>
-        <v>0.20836274065604599</v>
+        <v>0.2083627406574422</v>
       </c>
       <c r="P29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,P$9))</f>
-        <v>0.22410113154449718</v>
+        <v>0.22410113154599642</v>
       </c>
       <c r="Q29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,Q$9))</f>
-        <v>0.23983952243294837</v>
+        <v>0.2398395224345542</v>
       </c>
       <c r="R29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,R$9))</f>
-        <v>0.25557791332139956</v>
+        <v>0.25557791332310842</v>
       </c>
       <c r="S29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,S$9))</f>
-        <v>0.27131630420985076</v>
+        <v>0.27131630421166619</v>
       </c>
       <c r="T29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,T$9))</f>
-        <v>0.28705469509830195</v>
+        <v>0.28705469510022041</v>
       </c>
       <c r="U29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,U$9))</f>
-        <v>0.30279308598675314</v>
+        <v>0.30279308598877819</v>
       </c>
       <c r="V29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,V$9))</f>
-        <v>0.31853147687520433</v>
+        <v>0.31853147687733596</v>
       </c>
       <c r="W29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,W$9))</f>
-        <v>0.33426986776365553</v>
+        <v>0.33426986776589374</v>
       </c>
       <c r="X29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,X$9))</f>
-        <v>0.35000825865210672</v>
+        <v>0.3500082586544444</v>
       </c>
       <c r="Y29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,Y$9))</f>
-        <v>0.36574664954055791</v>
+        <v>0.36574664954300218</v>
       </c>
       <c r="Z29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,Z$9))</f>
-        <v>0.381485040429002</v>
+        <v>0.38148504043155995</v>
       </c>
       <c r="AA29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AA$9))</f>
-        <v>0.39722343131745319</v>
+        <v>0.39722343132011773</v>
       </c>
       <c r="AB29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AB$9))</f>
-        <v>0.41296182220590438</v>
+        <v>0.41296182220866839</v>
       </c>
       <c r="AC29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AC$9))</f>
-        <v>0.42870021309435558</v>
+        <v>0.42870021309722617</v>
       </c>
       <c r="AD29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AD$9))</f>
-        <v>0.44443860398280677</v>
+        <v>0.44443860398578394</v>
       </c>
       <c r="AE29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AE$9))</f>
-        <v>0.46017699487125796</v>
+        <v>0.46017699487434172</v>
       </c>
       <c r="AF29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AF$9))</f>
-        <v>0.47591538575970915</v>
+        <v>0.47591538576289238</v>
       </c>
       <c r="AG29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AG$9))</f>
-        <v>0.49165377664816035</v>
+        <v>0.49165377665145016</v>
       </c>
       <c r="AH29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AH$9))</f>
-        <v>0.50739216753661154</v>
+        <v>0.50739216754000793</v>
       </c>
       <c r="AI29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AI$9))</f>
-        <v>0.52313055842506273</v>
+        <v>0.52313055842856571</v>
       </c>
       <c r="AJ29">
         <f>IF($G29="s-curve",$E29+($F29-$E29)*$I$2/(1+EXP($I$3*(COUNT($I$9:AJ$9)+$I$4))),TREND($E29:$F29,$E$9:$F$9,AJ$9))</f>
-        <v>0.53886894931351392</v>
+        <v>0.53886894931712348</v>
       </c>
     </row>
     <row r="30" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -62731,7 +62731,7 @@
       <c r="D30" s="23"/>
       <c r="E30" s="26">
         <f>'SYVbT-passenger'!H3/SUM('SYVbT-passenger'!3:3)</f>
-        <v>1.0880490304811035E-4</v>
+        <v>1.088049030359405E-4</v>
       </c>
       <c r="F30" s="26">
         <v>0.05</v>
@@ -62742,115 +62742,115 @@
       </c>
       <c r="I30" s="22">
         <f t="shared" si="1"/>
-        <v>1.0880490304811035E-4</v>
+        <v>1.088049030359405E-4</v>
       </c>
       <c r="J30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,J$9))</f>
-        <v>8.4589900062574685E-4</v>
+        <v>8.4589900061375677E-4</v>
       </c>
       <c r="K30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,K$9))</f>
-        <v>1.0986614672101446E-3</v>
+        <v>1.0986614671982162E-3</v>
       </c>
       <c r="L30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,L$9))</f>
-        <v>1.4357606985839016E-3</v>
+        <v>1.4357606985720554E-3</v>
       </c>
       <c r="M30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,M$9))</f>
-        <v>1.8834940468798042E-3</v>
+        <v>1.883494046868067E-3</v>
       </c>
       <c r="N30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,N$9))</f>
-        <v>2.4749383943933924E-3</v>
+        <v>2.4749383943817997E-3</v>
       </c>
       <c r="O30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,O$9))</f>
-        <v>3.2506208959975401E-3</v>
+        <v>3.2506208959861365E-3</v>
       </c>
       <c r="P30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,P$9))</f>
-        <v>4.2583901305659581E-3</v>
+        <v>4.2583901305548004E-3</v>
       </c>
       <c r="Q30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,Q$9))</f>
-        <v>5.5517756937757106E-3</v>
+        <v>5.5517756937648686E-3</v>
       </c>
       <c r="R30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,R$9))</f>
-        <v>7.185924056708733E-3</v>
+        <v>7.1859240566982891E-3</v>
       </c>
       <c r="S30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,S$9))</f>
-        <v>9.2102323019346774E-3</v>
+        <v>9.210232301924727E-3</v>
       </c>
       <c r="T30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,T$9))</f>
-        <v>1.1657380089607801E-2</v>
+        <v>1.1657380089598447E-2</v>
       </c>
       <c r="U30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,U$9))</f>
-        <v>1.452987966045502E-2</v>
+        <v>1.4529879660446367E-2</v>
       </c>
       <c r="V30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,V$9))</f>
-        <v>1.7787435260511523E-2</v>
+        <v>1.7787435260503668E-2</v>
       </c>
       <c r="W30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,W$9))</f>
-        <v>2.1340376321765452E-2</v>
+        <v>2.1340376321758465E-2</v>
       </c>
       <c r="X30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,X$9))</f>
-        <v>2.5054402451524054E-2</v>
+        <v>2.5054402451517972E-2</v>
       </c>
       <c r="Y30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,Y$9))</f>
-        <v>2.8768428581282656E-2</v>
+        <v>2.876842858127748E-2</v>
       </c>
       <c r="Z30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,Z$9))</f>
-        <v>3.2321369642536582E-2</v>
+        <v>3.2321369642532273E-2</v>
       </c>
       <c r="AA30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AA$9))</f>
-        <v>3.5578925242593096E-2</v>
+        <v>3.5578925242589578E-2</v>
       </c>
       <c r="AB30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AB$9))</f>
-        <v>3.8451424813440313E-2</v>
+        <v>3.8451424813437496E-2</v>
       </c>
       <c r="AC30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AC$9))</f>
-        <v>4.0898572601113438E-2</v>
+        <v>4.0898572601111217E-2</v>
       </c>
       <c r="AD30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AD$9))</f>
-        <v>4.2922880846339384E-2</v>
+        <v>4.2922880846337656E-2</v>
       </c>
       <c r="AE30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AE$9))</f>
-        <v>4.4557029209272403E-2</v>
+        <v>4.4557029209271078E-2</v>
       </c>
       <c r="AF30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AF$9))</f>
-        <v>4.5850414772482161E-2</v>
+        <v>4.5850414772481148E-2</v>
       </c>
       <c r="AG30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AG$9))</f>
-        <v>4.6858184007050573E-2</v>
+        <v>4.6858184007049809E-2</v>
       </c>
       <c r="AH30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AH$9))</f>
-        <v>4.7633866508654726E-2</v>
+        <v>4.763386650865415E-2</v>
       </c>
       <c r="AI30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AI$9))</f>
-        <v>4.822531085616831E-2</v>
+        <v>4.822531085616788E-2</v>
       </c>
       <c r="AJ30">
         <f>IF($G30="s-curve",$E30+($F30-$E30)*$I$2/(1+EXP($I$3*(COUNT($I$9:AJ$9)+$I$4))),TREND($E30:$F30,$E$9:$F$9,AJ$9))</f>
-        <v>4.8673044204464208E-2</v>
+        <v>4.8673044204463882E-2</v>
       </c>
     </row>
     <row r="31" spans="1:36" x14ac:dyDescent="0.25">
@@ -65563,7 +65563,7 @@
       </c>
       <c r="E52" s="22">
         <f>'SYVbT-passenger'!B5/SUM('SYVbT-passenger'!B5:H5)</f>
-        <v>0.93664816809218165</v>
+        <v>0.93664816810144857</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -65574,115 +65574,115 @@
       </c>
       <c r="I52" s="22">
         <f t="shared" si="2"/>
-        <v>0.93664816809218165</v>
+        <v>0.93664816810144857</v>
       </c>
       <c r="J52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,J$9))</f>
-        <v>0.93758413006461472</v>
+        <v>0.93758413007374464</v>
       </c>
       <c r="K52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,K$9))</f>
-        <v>0.93790508780604664</v>
+        <v>0.93790508781512971</v>
       </c>
       <c r="L52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,L$9))</f>
-        <v>0.93833313635851656</v>
+        <v>0.93833313636753701</v>
       </c>
       <c r="M52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,M$9))</f>
-        <v>0.93890166809574294</v>
+        <v>0.93890166810468023</v>
       </c>
       <c r="N52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,N$9))</f>
-        <v>0.93965268403780833</v>
+        <v>0.93965268404663582</v>
       </c>
       <c r="O52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,O$9))</f>
-        <v>0.94063764555977569</v>
+        <v>0.94063764556845908</v>
       </c>
       <c r="P52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,P$9))</f>
-        <v>0.94191731077978458</v>
+        <v>0.94191731078828078</v>
       </c>
       <c r="Q52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,Q$9))</f>
-        <v>0.94355965157024346</v>
+        <v>0.94355965157849941</v>
       </c>
       <c r="R52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,R$9))</f>
-        <v>0.94563469291170243</v>
+        <v>0.94563469291965474</v>
       </c>
       <c r="S52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,S$9))</f>
-        <v>0.94820515921205761</v>
+        <v>0.94820515921963411</v>
       </c>
       <c r="T52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,T$9))</f>
-        <v>0.95131254709877777</v>
+        <v>0.95131254710589963</v>
       </c>
       <c r="U52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,U$9))</f>
-        <v>0.95496004661475364</v>
+        <v>0.95496004662134204</v>
       </c>
       <c r="V52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,V$9))</f>
-        <v>0.95909649021776056</v>
+        <v>0.95909649022374377</v>
       </c>
       <c r="W52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,W$9))</f>
-        <v>0.96360801423424369</v>
+        <v>0.96360801423956699</v>
       </c>
       <c r="X52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,X$9))</f>
-        <v>0.96832408404609083</v>
+        <v>0.96832408405072434</v>
       </c>
       <c r="Y52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,Y$9))</f>
-        <v>0.97304015385793796</v>
+        <v>0.97304015386188158</v>
       </c>
       <c r="Z52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,Z$9))</f>
-        <v>0.9775516778744211</v>
+        <v>0.97755167787770481</v>
       </c>
       <c r="AA52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AA$9))</f>
-        <v>0.98168812147742801</v>
+        <v>0.98168812148010653</v>
       </c>
       <c r="AB52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AB$9))</f>
-        <v>0.98533562099340388</v>
+        <v>0.98533562099554894</v>
       </c>
       <c r="AC52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AC$9))</f>
-        <v>0.98844300888012404</v>
+        <v>0.98844300888181458</v>
       </c>
       <c r="AD52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AD$9))</f>
-        <v>0.99101347518047922</v>
+        <v>0.99101347518179383</v>
       </c>
       <c r="AE52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AE$9))</f>
-        <v>0.99308851652193819</v>
+        <v>0.99308851652294916</v>
       </c>
       <c r="AF52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AF$9))</f>
-        <v>0.99473085731239708</v>
+        <v>0.99473085731316779</v>
       </c>
       <c r="AG52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AG$9))</f>
-        <v>0.99601052253240596</v>
+        <v>0.9960105225329895</v>
       </c>
       <c r="AH52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AH$9))</f>
-        <v>0.99699548405437333</v>
+        <v>0.99699548405481275</v>
       </c>
       <c r="AI52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AI$9))</f>
-        <v>0.99774649999643872</v>
+        <v>0.99774649999676845</v>
       </c>
       <c r="AJ52">
         <f>IF($G52="s-curve",$E52+($F52-$E52)*$I$2/(1+EXP($I$3*(COUNT($I$9:AJ$9)+$I$4))),TREND($E52:$F52,$E$9:$F$9,AJ$9))</f>
-        <v>0.99831503173366509</v>
+        <v>0.99831503173391156</v>
       </c>
     </row>
     <row r="53" spans="1:36" x14ac:dyDescent="0.25">
@@ -65945,7 +65945,7 @@
       </c>
       <c r="E55" s="22">
         <f>1-E52</f>
-        <v>6.3351831907818346E-2</v>
+        <v>6.3351831898551425E-2</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -65956,111 +65956,111 @@
       </c>
       <c r="I55" s="22">
         <f t="shared" si="2"/>
-        <v>6.3351831907818346E-2</v>
+        <v>6.3351831898551425E-2</v>
       </c>
       <c r="J55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,J$9))</f>
-        <v>6.3351831907809242E-2</v>
+        <v>6.3351831898543765E-2</v>
       </c>
       <c r="K55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,K$9))</f>
-        <v>9.9376761449818218E-2</v>
+        <v>9.9376761440908012E-2</v>
       </c>
       <c r="L55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,L$9))</f>
-        <v>0.13540169099182719</v>
+        <v>0.13540169098327226</v>
       </c>
       <c r="M55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,M$9))</f>
-        <v>0.17142662053383617</v>
+        <v>0.17142662052563651</v>
       </c>
       <c r="N55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,N$9))</f>
-        <v>0.20745155007584515</v>
+        <v>0.20745155006800076</v>
       </c>
       <c r="O55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,O$9))</f>
-        <v>0.24347647961785412</v>
+        <v>0.243476479610365</v>
       </c>
       <c r="P55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,P$9))</f>
-        <v>0.2795014091598631</v>
+        <v>0.27950140915272925</v>
       </c>
       <c r="Q55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,Q$9))</f>
-        <v>0.31552633870185787</v>
+        <v>0.3155263386950935</v>
       </c>
       <c r="R55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,R$9))</f>
-        <v>0.35155126824386684</v>
+        <v>0.35155126823745775</v>
       </c>
       <c r="S55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,S$9))</f>
-        <v>0.38757619778587582</v>
+        <v>0.387576197779822</v>
       </c>
       <c r="T55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,T$9))</f>
-        <v>0.4236011273278848</v>
+        <v>0.42360112732218624</v>
       </c>
       <c r="U55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,U$9))</f>
-        <v>0.45962605686989377</v>
+        <v>0.45962605686455049</v>
       </c>
       <c r="V55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,V$9))</f>
-        <v>0.49565098641190275</v>
+        <v>0.49565098640691474</v>
       </c>
       <c r="W55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,W$9))</f>
-        <v>0.53167591595391173</v>
+        <v>0.53167591594927899</v>
       </c>
       <c r="X55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,X$9))</f>
-        <v>0.56770084549590649</v>
+        <v>0.56770084549164324</v>
       </c>
       <c r="Y55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,Y$9))</f>
-        <v>0.60372577503791547</v>
+        <v>0.60372577503400748</v>
       </c>
       <c r="Z55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,Z$9))</f>
-        <v>0.63975070457992445</v>
+        <v>0.63975070457635752</v>
       </c>
       <c r="AA55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AA$9))</f>
-        <v>0.67577563412193342</v>
+        <v>0.67577563411872177</v>
       </c>
       <c r="AB55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AB$9))</f>
-        <v>0.7118005636639424</v>
+        <v>0.71180056366108602</v>
       </c>
       <c r="AC55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AC$9))</f>
-        <v>0.74782549320595137</v>
+        <v>0.74782549320345026</v>
       </c>
       <c r="AD55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AD$9))</f>
-        <v>0.78385042274796035</v>
+        <v>0.78385042274581451</v>
       </c>
       <c r="AE55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AE$9))</f>
-        <v>0.81987535228995512</v>
+        <v>0.81987535228817876</v>
       </c>
       <c r="AF55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AF$9))</f>
-        <v>0.85590028183196409</v>
+        <v>0.85590028183054301</v>
       </c>
       <c r="AG55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AG$9))</f>
-        <v>0.89192521137397307</v>
+        <v>0.89192521137290726</v>
       </c>
       <c r="AH55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AH$9))</f>
-        <v>0.92795014091598205</v>
+        <v>0.9279501409152715</v>
       </c>
       <c r="AI55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AI$9))</f>
-        <v>0.96397507045799102</v>
+        <v>0.96397507045763575</v>
       </c>
       <c r="AJ55">
         <f>IF($G55="s-curve",$E55+($F55-$E55)*$I$2/(1+EXP($I$3*(COUNT($I$9:AJ$9)+$I$4))),TREND($E55:$F55,$E$9:$F$9,AJ$9))</f>

</xml_diff>